<commit_message>
chore: init vault scaffolding 3
</commit_message>
<xml_diff>
--- a/tracker/Vault-Tracker.xlsx
+++ b/tracker/Vault-Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1694e94ce71b8319/Documents/aws-project-vault/tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="127" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{908536C6-8248-43CD-9899-5B52E3382F35}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4E0F6E0A-CAC8-4200-935A-CF6F2F72C4A3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>Module #</t>
   </si>
@@ -63,19 +63,100 @@
   </si>
   <si>
     <t>Proof links</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>us-east-1</t>
+  </si>
+  <si>
+    <t>Next action</t>
+  </si>
+  <si>
+    <t>Start Here</t>
+  </si>
+  <si>
+    <t>Setup &amp; Tools</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Week</t>
+  </si>
+  <si>
+    <t>Velocity (min/week)</t>
+  </si>
+  <si>
+    <t>Completion %</t>
+  </si>
+  <si>
+    <t>02-23-2026 -- 2:36 -- everything is set up.</t>
+  </si>
+  <si>
+    <t>Progress Tracker &amp; Learning Management</t>
+  </si>
+  <si>
+    <t>How to Use This Vault Effectively</t>
+  </si>
+  <si>
+    <t>Not started</t>
+  </si>
+  <si>
+    <t>Serverless URL Shortener</t>
+  </si>
+  <si>
+    <t>Personal File Backup System</t>
+  </si>
+  <si>
+    <t>Secure Notes App</t>
+  </si>
+  <si>
+    <t>Real-Time Log Monitoring Dashboard</t>
+  </si>
+  <si>
+    <t>Automated Resume Website</t>
+  </si>
+  <si>
+    <t>IoT Sensor Data Pipeline</t>
+  </si>
+  <si>
+    <t>Multi-Region Static Website</t>
+  </si>
+  <si>
+    <t>Automated Image Processing</t>
+  </si>
+  <si>
+    <t>Cost Optimization Bot</t>
+  </si>
+  <si>
+    <t>Disaster Recovery Simulation</t>
+  </si>
+  <si>
+    <t>aws-project-vault\project00-start-here\screenshots</t>
+  </si>
+  <si>
+    <t>Score</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.35"/>
+      <color rgb="FFEB5757"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -98,8 +179,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -434,10 +516,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B7516CF-FA71-4510-B2CE-909010B84E70}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" customWidth="1"/>
+    <col min="3" max="3" width="32.109375" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="8" max="8" width="16.5546875" customWidth="1"/>
+    <col min="9" max="9" width="33.44140625" customWidth="1"/>
+    <col min="10" max="10" width="17.109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -465,8 +559,232 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2">
+        <v>50</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2">
+        <v>100</v>
+      </c>
+      <c r="L2" s="1" t="str">
+        <f>IFERROR("Wk "&amp;TEXT(DATEVALUE(LEFT(H2,10)),"YYYY")&amp;"-"&amp;TEXT(DATEVALUE(LEFT(H2,L210)),"WW"),"")</f>
+        <v/>
+      </c>
+      <c r="M2" s="1">
+        <f ca="1">SUMIFS($D:$D,$H:$H,"&gt;="&amp;TODAY()-14,$H:$H,"&lt;="&amp;TODAY())</f>
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <f>IF(COUNTIF($C:$C,"&lt;&gt;")=0,"",COUNTIF($C:$C,"Done")/COUNTIF($C:$C,"&lt;&gt;"))</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3">
+        <v>100</v>
+      </c>
+      <c r="M3" s="1">
+        <f ca="1">SUMIFS($D:$D,$H:$H,"&gt;="&amp;TODAY()-14,$H:$H,"&lt;="&amp;TODAY())</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <v>30</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C15" xr:uid="{209531A9-0B50-4602-9185-0821BA45A4F3}">
+      <formula1>"Not started,In Progress,Blocked,Done"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
url-shortener: created and deployed POST method
</commit_message>
<xml_diff>
--- a/tracker/Vault-Tracker.xlsx
+++ b/tracker/Vault-Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1694e94ce71b8319/Documents/aws-project-vault/tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="127" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{908536C6-8248-43CD-9899-5B52E3382F35}"/>
+  <xr:revisionPtr revIDLastSave="162" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{149BBE3B-9EDA-451F-B4C6-9CB20CBF1288}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4E0F6E0A-CAC8-4200-935A-CF6F2F72C4A3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
   <si>
     <t>Module #</t>
   </si>
@@ -92,9 +92,6 @@
     <t>Completion %</t>
   </si>
   <si>
-    <t>02-23-2026 -- 2:36 -- everything is set up.</t>
-  </si>
-  <si>
     <t>Progress Tracker &amp; Learning Management</t>
   </si>
   <si>
@@ -138,6 +135,12 @@
   </si>
   <si>
     <t>Score</t>
+  </si>
+  <si>
+    <t>2026-02-23 -- 2:36 -- everything is set up.</t>
+  </si>
+  <si>
+    <t>Create DynamoDB Table</t>
   </si>
 </sst>
 </file>
@@ -529,6 +532,8 @@
     <col min="8" max="8" width="16.5546875" customWidth="1"/>
     <col min="9" max="9" width="33.44140625" customWidth="1"/>
     <col min="10" max="10" width="17.109375" customWidth="1"/>
+    <col min="11" max="11" width="19.21875" customWidth="1"/>
+    <col min="12" max="12" width="24.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -560,7 +565,7 @@
         <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K1" t="s">
         <v>11</v>
@@ -589,17 +594,17 @@
         <v>50</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="I2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J2">
         <v>100</v>
       </c>
       <c r="L2" s="1" t="str">
-        <f>IFERROR("Wk "&amp;TEXT(DATEVALUE(LEFT(H2,10)),"YYYY")&amp;"-"&amp;TEXT(DATEVALUE(LEFT(H2,L210)),"WW"),"")</f>
-        <v/>
+        <f>IFERROR("Wk "&amp;TEXT(DATEVALUE(LEFT(H2,10)),"YYYY")&amp;"-"&amp;TEXT(DATEVALUE(LEFT(H2,10)),"WW"),"")</f>
+        <v>Wk 2026-WW</v>
       </c>
       <c r="M2" s="1">
         <f ca="1">SUMIFS($D:$D,$H:$H,"&gt;="&amp;TODAY()-14,$H:$H,"&lt;="&amp;TODAY())</f>
@@ -607,7 +612,7 @@
       </c>
       <c r="N2">
         <f>IF(COUNTIF($C:$C,"&lt;&gt;")=0,"",COUNTIF($C:$C,"Done")/COUNTIF($C:$C,"&lt;&gt;"))</f>
-        <v>0.2</v>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -627,17 +632,25 @@
         <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="I3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J3">
         <v>100</v>
       </c>
+      <c r="L3" s="1" t="str">
+        <f>IFERROR("Wk "&amp;TEXT(DATEVALUE(LEFT(H3,10)),"YYYY")&amp;"-"&amp;TEXT(DATEVALUE(LEFT(H3,10)),"WW"),"")</f>
+        <v>Wk 2026-WW</v>
+      </c>
       <c r="M3" s="1">
         <f ca="1">SUMIFS($D:$D,$H:$H,"&gt;="&amp;TODAY()-14,$H:$H,"&lt;="&amp;TODAY())</f>
         <v>0</v>
+      </c>
+      <c r="N3">
+        <f t="shared" ref="N3:N15" si="0">IF(COUNTIF($C:$C,"&lt;&gt;")=0,"",COUNTIF($C:$C,"Done")/COUNTIF($C:$C,"&lt;&gt;"))</f>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -645,7 +658,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
@@ -653,8 +666,26 @@
       <c r="D4">
         <v>30</v>
       </c>
-      <c r="H4">
-        <v>2</v>
+      <c r="H4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4">
+        <v>100</v>
+      </c>
+      <c r="L4" s="1" t="str">
+        <f t="shared" ref="L4:L15" si="1">IFERROR("Wk "&amp;TEXT(DATEVALUE(LEFT(H4,10)),"YYYY")&amp;"-"&amp;TEXT(DATEVALUE(LEFT(H4,10)),"WW"),"")</f>
+        <v>Wk 2026-WW</v>
+      </c>
+      <c r="M4" s="1">
+        <f t="shared" ref="M4:M15" ca="1" si="2">SUMIFS($D:$D,$H:$H,"&gt;="&amp;TODAY()-14,$H:$H,"&lt;="&amp;TODAY())</f>
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -662,10 +693,34 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>14</v>
+      </c>
+      <c r="D5">
+        <v>30</v>
+      </c>
+      <c r="H5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J5">
+        <v>100</v>
+      </c>
+      <c r="L5" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>Wk 2026-WW</v>
+      </c>
+      <c r="M5" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -673,10 +728,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>9</v>
+      </c>
+      <c r="K6" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M6" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -684,10 +754,22 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="L7" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M7" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -695,10 +777,22 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="L8" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M8" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -706,10 +800,22 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="L9" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M9" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -717,10 +823,22 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="L10" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M10" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -728,10 +846,22 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="L11" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M11" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -739,10 +869,22 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="L12" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M12" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
@@ -750,10 +892,22 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="L13" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M13" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -761,10 +915,22 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="L14" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M14" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -772,10 +938,22 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="L15" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M15" s="1">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="0"/>
+        <v>0.26666666666666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Project 2 notes update
</commit_message>
<xml_diff>
--- a/tracker/Vault-Tracker.xlsx
+++ b/tracker/Vault-Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1694e94ce71b8319/Documents/aws-project-vault/tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="175" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA04A562-88E4-4245-A558-BEBB5A27D386}"/>
+  <xr:revisionPtr revIDLastSave="179" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34C9585C-F598-4182-AB3F-A59F5A82F6AB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4E0F6E0A-CAC8-4200-935A-CF6F2F72C4A3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
   <si>
     <t>Module #</t>
   </si>
@@ -146,7 +146,10 @@
     <t>In Progress</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-02-25 -- 10:50 -- </t>
+    <t>2026-02-25 - 120 min - Project 2 Core path worked. / Security Enhancements</t>
+  </si>
+  <si>
+    <t>aws-project-vault\02-file-backup-system\screenshots</t>
   </si>
 </sst>
 </file>
@@ -781,6 +784,12 @@
       <c r="H7" t="s">
         <v>36</v>
       </c>
+      <c r="I7" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7">
+        <v>89</v>
+      </c>
       <c r="L7" s="1" t="str">
         <f t="shared" si="1"/>
         <v>Wk 2026-WW</v>

</xml_diff>

<commit_message>
Complete core of project 3
</commit_message>
<xml_diff>
--- a/tracker/Vault-Tracker.xlsx
+++ b/tracker/Vault-Tracker.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1694e94ce71b8319/Documents/aws-project-vault/tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="183" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF38A6F8-64EB-43F9-8FBD-51C0072B7CE6}"/>
+  <xr:revisionPtr revIDLastSave="186" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFD784D4-117E-4588-8CDE-CDB3172BBEEB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4E0F6E0A-CAC8-4200-935A-CF6F2F72C4A3}"/>
+    <workbookView xWindow="2556" yWindow="2172" windowWidth="17280" windowHeight="8820" xr2:uid="{4E0F6E0A-CAC8-4200-935A-CF6F2F72C4A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="39">
   <si>
     <t>Module #</t>
   </si>
@@ -150,6 +151,9 @@
   </si>
   <si>
     <t>aws-project-vault\02-file-backup-system\screenshots</t>
+  </si>
+  <si>
+    <t>aws-project-vault\03-secure-notes-app\screenshots</t>
   </si>
 </sst>
 </file>
@@ -209,6 +213,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -810,7 +818,13 @@
         <v>35</v>
       </c>
       <c r="D8">
-        <v>120</v>
+        <v>275</v>
+      </c>
+      <c r="I8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J8">
+        <v>89</v>
       </c>
       <c r="L8" s="1" t="str">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
created website for project 5
</commit_message>
<xml_diff>
--- a/tracker/Vault-Tracker.xlsx
+++ b/tracker/Vault-Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1694e94ce71b8319/Documents/aws-project-vault/tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="191" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{968F08E9-4981-4B45-AA0F-AC4B06D32F0F}"/>
+  <xr:revisionPtr revIDLastSave="195" documentId="8_{9FFB97A3-CFAA-4478-A377-388F42B319C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1415A8ED-5A0A-436B-9415-A407099C35EC}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="2172" windowWidth="17280" windowHeight="8820" xr2:uid="{4E0F6E0A-CAC8-4200-935A-CF6F2F72C4A3}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
   <si>
     <t>Module #</t>
   </si>
@@ -157,6 +156,9 @@
   </si>
   <si>
     <t>2026-03-03 - 120 min -</t>
+  </si>
+  <si>
+    <t>aws-project-vault\04-real-time-log-monitoring-dashboard\screenshots</t>
   </si>
 </sst>
 </file>
@@ -632,7 +634,7 @@
       </c>
       <c r="N2">
         <f>IF(COUNTIF($C:$C,"&lt;&gt;")=0,"",COUNTIF($C:$C,"Done")/COUNTIF($C:$C,"&lt;&gt;"))</f>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -670,7 +672,7 @@
       </c>
       <c r="N3">
         <f t="shared" ref="N3:N15" si="0">IF(COUNTIF($C:$C,"&lt;&gt;")=0,"",COUNTIF($C:$C,"Done")/COUNTIF($C:$C,"&lt;&gt;"))</f>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -705,7 +707,7 @@
       </c>
       <c r="N4">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -740,7 +742,7 @@
       </c>
       <c r="N5">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -775,7 +777,7 @@
       </c>
       <c r="N6">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -807,7 +809,7 @@
       </c>
       <c r="N7">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -839,7 +841,7 @@
       </c>
       <c r="N8">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -850,13 +852,19 @@
         <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="D9">
         <v>120</v>
       </c>
       <c r="H9" t="s">
         <v>39</v>
+      </c>
+      <c r="I9" t="s">
+        <v>40</v>
+      </c>
+      <c r="J9">
+        <v>89</v>
       </c>
       <c r="L9" s="1" t="str">
         <f t="shared" si="1"/>
@@ -868,7 +876,7 @@
       </c>
       <c r="N9">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -879,7 +887,7 @@
         <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="L10" s="1" t="str">
         <f t="shared" si="1"/>
@@ -891,7 +899,7 @@
       </c>
       <c r="N10">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -914,7 +922,7 @@
       </c>
       <c r="N11">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -937,7 +945,7 @@
       </c>
       <c r="N12">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
@@ -960,7 +968,7 @@
       </c>
       <c r="N13">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -983,7 +991,7 @@
       </c>
       <c r="N14">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -1006,7 +1014,7 @@
       </c>
       <c r="N15">
         <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>